<commit_message>
feat(obstacle-count-data-driven): story-001 障碍数量迁入 CellGlobal.obstacleCount
ObstacleGenerator.Count 硬编码改为运行时读 DataRegistry.Instance.Global.ObstacleCount；
新增 GlobalSpec 出口，CellLubanLoader/CellContentSeed 补齐 Luban 表读取与回落默认值；
CellGlobal 表新增 obstacleCount 列（重跑 gen_all.py + Luban codegen 生成，未手改生成产物）。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#CellGlobal-全局常量.xlsx
+++ b/Configs/GameConfig/Datas/cell/#CellGlobal-全局常量.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,6 +547,11 @@
           <t>synergyBonusCap</t>
         </is>
       </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>obstacleCount</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -679,6 +684,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -809,6 +819,11 @@
       <c r="Z3" t="inlineStr">
         <is>
           <t>联动加成上限</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>局内静态障碍数量</t>
         </is>
       </c>
     </row>
@@ -889,6 +904,9 @@
       <c r="Z4" t="n">
         <v>1.5</v>
       </c>
+      <c r="AA4" t="n">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>